<commit_message>
Documentation pack: release figures aligned with the release verification of 04 October 2026 (UAT 433 steps, rehearsal 52 checks, 1,113 backend and 175 front-end tests, 629 test cases, migrations to 0331, 8 roles, 74 upload templates, user manual 1.2); packages B and G recorded as merged; 15 documents rebuilt
</commit_message>
<xml_diff>
--- a/docs/package/04_Onboarding_and_Go_Live/BrokerVerse_Security_Due_Diligence_Questionnaire.xlsx
+++ b/docs/package/04_Onboarding_and_Go_Live/BrokerVerse_Security_Due_Diligence_Questionnaire.xlsx
@@ -3582,7 +3582,7 @@
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>634 backend business-rule tests (03 October 2026), 43 front-end tests, a 371-step end-to-end UAT cycle with one user per role</t>
+          <t>1,113 backend tests in 104 files and 175 front-end tests in 33 suites (04 October 2026, merged release), a 433-step end-to-end UAT cycle with one user per role and a 52-check go-live rehearsal</t>
         </is>
       </c>
       <c r="F90" s="2" t="inlineStr">
@@ -4564,7 +4564,7 @@
       </c>
       <c r="E119" s="2" t="inlineStr">
         <is>
-          <t>AIS compliance checklist; PRCM; TSR with 497 test cases and traceability to automated tests</t>
+          <t>AIS compliance checklist; PRCM; TSR with 629 test cases and traceability to automated tests</t>
         </is>
       </c>
       <c r="F119" s="2" t="inlineStr">

</xml_diff>